<commit_message>
Re-theme business plan workbook to navy/teal/gold
Matches the color update just made to the app: swaps the purple
header/section fills and title font for the same navy-teal-gold
palette, so the two deliverables read as one product.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014M6j9p1JE8CUXwus4sEArJ
</commit_message>
<xml_diff>
--- a/docs/Mystic_Companion_Business_Plan.xlsx
+++ b/docs/Mystic_Companion_Business_Plan.xlsx
@@ -1537,7 +1537,7 @@
     <font>
       <b val="true"/>
       <sz val="18"/>
-      <color rgb="FF4B1F80"/>
+      <color rgb="FF0F3A4D"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1545,7 +1545,7 @@
     <font>
       <i val="true"/>
       <sz val="11"/>
-      <color rgb="FF6B6375"/>
+      <color rgb="FF5C7A8A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1614,20 +1614,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7C3AED"/>
-        <bgColor rgb="FF993366"/>
+        <fgColor rgb="FF1C7488"/>
+        <bgColor rgb="FF12566A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7F5FB"/>
+        <fgColor rgb="FFF3F7F9"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4B1F80"/>
-        <bgColor rgb="FF660066"/>
+        <fgColor rgb="FF12566A"/>
+        <bgColor rgb="FF0F3A4D"/>
       </patternFill>
     </fill>
     <fill>
@@ -1638,14 +1638,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDE7F6"/>
-        <bgColor rgb="FFF7F5FB"/>
+        <fgColor rgb="FFDCEEF2"/>
+        <bgColor rgb="FFF3F7F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5C451"/>
-        <bgColor rgb="FFFFCC00"/>
+        <fgColor rgb="FFF2D89B"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -1892,13 +1892,13 @@
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF1C7488"/>
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF7C3AED"/>
-      <rgbColor rgb="FFF7F5FB"/>
-      <rgbColor rgb="FFEDE7F6"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFF3F7F9"/>
+      <rgbColor rgb="FFDCEEF2"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1909,7 +1909,7 @@
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF12566A"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
@@ -1918,22 +1918,22 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF5C451"/>
+      <rgbColor rgb="FFF2D89B"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF6B6375"/>
+      <rgbColor rgb="FF5C7A8A"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF0F3A4D"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF4B1F80"/>
+      <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>

</xml_diff>